<commit_message>
renamed Date to date
</commit_message>
<xml_diff>
--- a/data/Ebola-2026-manual-data.xlsx
+++ b/data/Ebola-2026-manual-data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Ebola-2026\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72A06765-04D2-44F5-9B69-CFCC12A9F0C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6268B50-CDB2-456A-B71F-BB860C5B541D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,9 +33,6 @@
     <t>Province</t>
   </si>
   <si>
-    <t>Date</t>
-  </si>
-  <si>
     <t>DRC health zone</t>
   </si>
   <si>
@@ -49,6 +46,9 @@
   </si>
   <si>
     <t>DRC</t>
+  </si>
+  <si>
+    <t>date</t>
   </si>
 </sst>
 </file>
@@ -115,7 +115,7 @@
     <tableColumn id="1" xr3:uid="{55B41B7D-F471-4598-B55D-30D0C294BAD5}" name="Country"/>
     <tableColumn id="5" xr3:uid="{117FAE87-256C-4E93-AD73-A0020763145A}" name="Province"/>
     <tableColumn id="2" xr3:uid="{E46D03F0-7BC0-45FB-B0A3-DF8A25685268}" name="DRC health zone"/>
-    <tableColumn id="3" xr3:uid="{C0CA5BF8-A724-4962-A17F-A952CB6E6CC8}" name="Date" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{C0CA5BF8-A724-4962-A17F-A952CB6E6CC8}" name="date" dataDxfId="0"/>
     <tableColumn id="4" xr3:uid="{F0291790-FC35-4FEE-ADD2-161583682016}" name="Cumulative Confirmed Cases"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -396,16 +396,16 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E1" t="s">
         <v>0</v>
@@ -413,13 +413,13 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
         <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
       </c>
       <c r="D2" s="1">
         <v>46165</v>
@@ -430,13 +430,13 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
         <v>4</v>
-      </c>
-      <c r="C3" t="s">
-        <v>5</v>
       </c>
       <c r="D3" s="1">
         <v>46166</v>
@@ -447,13 +447,13 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
         <v>4</v>
-      </c>
-      <c r="C4" t="s">
-        <v>5</v>
       </c>
       <c r="D4" s="1">
         <v>46167</v>
@@ -464,13 +464,13 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
         <v>4</v>
-      </c>
-      <c r="C5" t="s">
-        <v>5</v>
       </c>
       <c r="D5" s="1">
         <v>46168</v>
@@ -481,13 +481,13 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" t="s">
         <v>4</v>
-      </c>
-      <c r="C6" t="s">
-        <v>5</v>
       </c>
       <c r="D6" s="1">
         <v>46169</v>

</xml_diff>

<commit_message>
updated to reflect shapefile in source project
Country changed from DRC to COD (ISO3)
</commit_message>
<xml_diff>
--- a/data/Ebola-2026-manual-data.xlsx
+++ b/data/Ebola-2026-manual-data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Ebola-2026\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C944D97-B82B-450A-8269-6B7D2068CDB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8231357-5F18-4F10-892B-1C84A5B165B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,10 +39,10 @@
     <t>Country</t>
   </si>
   <si>
-    <t>DRC</t>
-  </si>
-  <si>
     <t>NA</t>
+  </si>
+  <si>
+    <t>COD</t>
   </si>
 </sst>
 </file>
@@ -392,13 +392,13 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>